<commit_message>
Full Triplet + Debug
Full triplet functionality added, de some bugs, and more.

Features:
 - Fully implemented Triplet code functionality. Has separate window (similar to that of CA cycle) with custom settings. Also integrates with source vial position with options to draw, simulate, or ignore content in source vial.
 - Gathered position for all 24 cell positions (except 6A, out of reach of robot).

GUI Changes:
 - Added new color scheme and distinct indicator for QUEUED, RUNNING, FAILED, and COMPLETED tests on UI.
 - Log Notes:  functionality to add notes to respective column in plate log for each cell (sorted by the current plate ID and cell position)
 - Clear Status: Clears all status indicators and resets grid

Bugs Squashed:
 - CV held at desired starting voltage for set time length (default: 2s) before executing CV to prevent unwanted current spikes
 - Cleaned GUI-related bugs with unwanted window expansion (not all cases yet discovered).
</commit_message>
<xml_diff>
--- a/MainProject/src/main/res/bumps/1413_1.xlsx
+++ b/MainProject/src/main/res/bumps/1413_1.xlsx
@@ -1907,4 +1907,282 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010085E7130ED883394FB144BCB9223171D8" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="c75b2c9d0baddedb5d5c9ac2f1c46d6f">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="a3154109-1d0c-437e-b5a5-e7f74c43baaa" xmlns:ns3="73ab24cd-13cc-4967-9ebd-27d2662a6de9" xmlns:ns4="efce84db-8738-4c7b-9bdc-65b9500871f6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d8c4dbb9606f2bd0ab8e2b49684024ea" ns2:_="" ns3:_="" ns4:_="">
+    <xsd:import namespace="a3154109-1d0c-437e-b5a5-e7f74c43baaa"/>
+    <xsd:import namespace="73ab24cd-13cc-4967-9ebd-27d2662a6de9"/>
+    <xsd:import namespace="efce84db-8738-4c7b-9bdc-65b9500871f6"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns4:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="a3154109-1d0c-437e-b5a5-e7f74c43baaa" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="c2d55d72-5afa-45f9-90b6-e0708aeee9a0" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="15" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="16" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="17" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="18" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="19" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="20" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="21" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceBillingMetadata" ma:index="22" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceLocation" ma:index="23" nillable="true" ma:displayName="Location" ma:description="" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="73ab24cd-13cc-4967-9ebd-27d2662a6de9" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="SharedWithUsers" ma:index="10" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:UserMulti">
+            <xsd:sequence>
+              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
+                <xsd:complexType>
+                  <xsd:sequence>
+                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
+                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
+                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
+                  </xsd:sequence>
+                </xsd:complexType>
+              </xsd:element>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithDetails" ma:index="11" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="efce84db-8738-4c7b-9bdc-65b9500871f6" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{51645941-b371-4c8e-94e2-de0bc4e067f8}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="73ab24cd-13cc-4967-9ebd-27d2662a6de9">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="efce84db-8738-4c7b-9bdc-65b9500871f6" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="a3154109-1d0c-437e-b5a5-e7f74c43baaa">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5960EBDC-F5EF-4DCE-BC73-6CA9E9C569D5}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3E68FA43-F0AA-4494-BB12-9448432B8F15}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{418A2DAA-2CEE-43DC-9B07-D2307F394652}"/>
 </file>
</xml_diff>